<commit_message>
Step1 TURN ON 변경, Step3 경과일 수정, RULE 업데이트 (2026-03-03)
</commit_message>
<xml_diff>
--- a/스케쥴 시트/★★이게진짜 Daily 종합사이트 스케줄★★.xlsx
+++ b/스케쥴 시트/★★이게진짜 Daily 종합사이트 스케줄★★.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\정동교\문서 자동화 TEST\커서 바이브코딩 자동화 관련\스케쥴 시트\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6462421D-C65C-4718-BF6F-8E96A09809ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A9B692B4-6B8E-44A1-946F-FE3114189269}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -2256,11 +2256,11 @@
       <alignment horizontal="left" vertical="center" shrinkToFit="1"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1" applyProtection="1">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="center"/>
       <protection locked="0"/>
     </xf>
@@ -2901,15 +2901,15 @@
     </row>
     <row r="2" spans="1:28" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A2" s="54"/>
-      <c r="B2" s="82" t="s">
+      <c r="B2" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="C2" s="82"/>
-      <c r="D2" s="82"/>
-      <c r="E2" s="82"/>
-      <c r="F2" s="82"/>
-      <c r="G2" s="82"/>
-      <c r="H2" s="82"/>
+      <c r="C2" s="81"/>
+      <c r="D2" s="81"/>
+      <c r="E2" s="81"/>
+      <c r="F2" s="81"/>
+      <c r="G2" s="81"/>
+      <c r="H2" s="81"/>
       <c r="I2" s="54"/>
       <c r="J2" s="54"/>
       <c r="K2" s="54"/>
@@ -5307,15 +5307,15 @@
     </row>
     <row r="49" spans="1:28" ht="32.25" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A49" s="54"/>
-      <c r="B49" s="82" t="s">
+      <c r="B49" s="81" t="s">
         <v>69</v>
       </c>
-      <c r="C49" s="82"/>
-      <c r="D49" s="82"/>
-      <c r="E49" s="82"/>
-      <c r="F49" s="82"/>
-      <c r="G49" s="82"/>
-      <c r="H49" s="82"/>
+      <c r="C49" s="81"/>
+      <c r="D49" s="81"/>
+      <c r="E49" s="81"/>
+      <c r="F49" s="81"/>
+      <c r="G49" s="81"/>
+      <c r="H49" s="81"/>
       <c r="I49" s="54"/>
       <c r="J49" s="54"/>
       <c r="K49" s="54"/>
@@ -7593,13 +7593,13 @@
     </row>
     <row r="92" spans="1:28" ht="42" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A92" s="54"/>
-      <c r="B92" s="81" t="s">
+      <c r="B92" s="82" t="s">
         <v>137</v>
       </c>
-      <c r="C92" s="81"/>
-      <c r="D92" s="81"/>
-      <c r="E92" s="81"/>
-      <c r="F92" s="81"/>
+      <c r="C92" s="82"/>
+      <c r="D92" s="82"/>
+      <c r="E92" s="82"/>
+      <c r="F92" s="82"/>
       <c r="G92" s="47" t="s">
         <v>289</v>
       </c>
@@ -9948,13 +9948,13 @@
     </row>
     <row r="138" spans="1:29" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A138" s="54"/>
-      <c r="B138" s="81" t="s">
+      <c r="B138" s="82" t="s">
         <v>182</v>
       </c>
-      <c r="C138" s="81"/>
-      <c r="D138" s="81"/>
-      <c r="E138" s="81"/>
-      <c r="F138" s="81"/>
+      <c r="C138" s="82"/>
+      <c r="D138" s="82"/>
+      <c r="E138" s="82"/>
+      <c r="F138" s="82"/>
       <c r="G138" s="47" t="s">
         <v>289</v>
       </c>
@@ -12176,13 +12176,13 @@
     </row>
     <row r="183" spans="1:29" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A183" s="54"/>
-      <c r="B183" s="81" t="s">
+      <c r="B183" s="82" t="s">
         <v>260</v>
       </c>
-      <c r="C183" s="81"/>
-      <c r="D183" s="81"/>
-      <c r="E183" s="81"/>
-      <c r="F183" s="81"/>
+      <c r="C183" s="82"/>
+      <c r="D183" s="82"/>
+      <c r="E183" s="82"/>
+      <c r="F183" s="82"/>
       <c r="G183" s="47" t="s">
         <v>289</v>
       </c>
@@ -13848,13 +13848,13 @@
     </row>
     <row r="228" spans="1:29" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A228" s="54"/>
-      <c r="B228" s="81" t="s">
+      <c r="B228" s="82" t="s">
         <v>259</v>
       </c>
-      <c r="C228" s="81"/>
-      <c r="D228" s="81"/>
-      <c r="E228" s="81"/>
-      <c r="F228" s="81"/>
+      <c r="C228" s="82"/>
+      <c r="D228" s="82"/>
+      <c r="E228" s="82"/>
+      <c r="F228" s="82"/>
       <c r="G228" s="47" t="s">
         <v>289</v>
       </c>
@@ -15444,13 +15444,13 @@
     </row>
     <row r="273" spans="1:29" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A273" s="54"/>
-      <c r="B273" s="81" t="s">
+      <c r="B273" s="82" t="s">
         <v>290</v>
       </c>
-      <c r="C273" s="81"/>
-      <c r="D273" s="81"/>
-      <c r="E273" s="81"/>
-      <c r="F273" s="81"/>
+      <c r="C273" s="82"/>
+      <c r="D273" s="82"/>
+      <c r="E273" s="82"/>
+      <c r="F273" s="82"/>
       <c r="G273" s="47" t="s">
         <v>289</v>
       </c>
@@ -17042,13 +17042,13 @@
     </row>
     <row r="318" spans="1:29" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A318" s="54"/>
-      <c r="B318" s="81" t="s">
+      <c r="B318" s="82" t="s">
         <v>291</v>
       </c>
-      <c r="C318" s="81"/>
-      <c r="D318" s="81"/>
-      <c r="E318" s="81"/>
-      <c r="F318" s="81"/>
+      <c r="C318" s="82"/>
+      <c r="D318" s="82"/>
+      <c r="E318" s="82"/>
+      <c r="F318" s="82"/>
       <c r="G318" s="47" t="s">
         <v>289</v>
       </c>
@@ -18638,13 +18638,13 @@
     </row>
     <row r="363" spans="1:29" ht="42" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A363" s="54"/>
-      <c r="B363" s="81" t="s">
+      <c r="B363" s="82" t="s">
         <v>292</v>
       </c>
-      <c r="C363" s="81"/>
-      <c r="D363" s="81"/>
-      <c r="E363" s="81"/>
-      <c r="F363" s="81"/>
+      <c r="C363" s="82"/>
+      <c r="D363" s="82"/>
+      <c r="E363" s="82"/>
+      <c r="F363" s="82"/>
       <c r="G363" s="47" t="s">
         <v>289</v>
       </c>
@@ -21676,24 +21676,24 @@
     </row>
   </sheetData>
   <mergeCells count="18">
+    <mergeCell ref="B395:H398"/>
+    <mergeCell ref="B273:F273"/>
+    <mergeCell ref="B305:H308"/>
+    <mergeCell ref="B318:F318"/>
+    <mergeCell ref="B350:H353"/>
+    <mergeCell ref="B363:F363"/>
+    <mergeCell ref="B215:H218"/>
+    <mergeCell ref="B260:H263"/>
+    <mergeCell ref="B170:H173"/>
+    <mergeCell ref="B138:F138"/>
+    <mergeCell ref="B183:F183"/>
+    <mergeCell ref="B228:F228"/>
     <mergeCell ref="B124:H127"/>
     <mergeCell ref="B2:H2"/>
     <mergeCell ref="B34:H37"/>
     <mergeCell ref="B49:H49"/>
     <mergeCell ref="B81:H84"/>
     <mergeCell ref="B92:F92"/>
-    <mergeCell ref="B215:H218"/>
-    <mergeCell ref="B260:H263"/>
-    <mergeCell ref="B170:H173"/>
-    <mergeCell ref="B138:F138"/>
-    <mergeCell ref="B183:F183"/>
-    <mergeCell ref="B228:F228"/>
-    <mergeCell ref="B395:H398"/>
-    <mergeCell ref="B273:F273"/>
-    <mergeCell ref="B305:H308"/>
-    <mergeCell ref="B318:F318"/>
-    <mergeCell ref="B350:H353"/>
-    <mergeCell ref="B363:F363"/>
   </mergeCells>
   <phoneticPr fontId="2" type="noConversion"/>
   <conditionalFormatting sqref="J93:K93 J139:K139 J184:K184 J229:K229">

</xml_diff>

<commit_message>
10차 세션 코드 반영: Step1~3 DB 연동 완료, db_init/db_export 추가, Step3 INSERT 수정
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/스케쥴 시트/★★이게진짜 Daily 종합사이트 스케줄★★.xlsx
+++ b/스케쥴 시트/★★이게진짜 Daily 종합사이트 스케줄★★.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\정동교\문서 자동화 TEST\커서 바이브코딩 자동화 관련\스케쥴 시트\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3E35E9A-7272-41AE-A408-483CA3937DBD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC8278E7-7912-4AE7-9D87-02E84B20AD3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="2565" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>